<commit_message>
Cache dictionary + formula "chronological" order
Added caching system to simulate Excel-like reactivity and speed up formula evaluation.
Improves performance, especially with long dependencies and circular-style formulas.

Removed all FFSS formulas from backend and started the process of reintroducing them in chronological order.
</commit_message>
<xml_diff>
--- a/backend/LPG testing/capex-fuels-BAU.xlsx
+++ b/backend/LPG testing/capex-fuels-BAU.xlsx
@@ -2118,25 +2118,25 @@
         <v>0.6504849465450439</v>
       </c>
       <c r="H10" s="11" t="n">
-        <v>0.7640156319949659</v>
+        <v>0.7577214998364629</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.7444297550238093</v>
+        <v>0.8206069930729</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>0.604700981496039</v>
+        <v>0.7537542136686143</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>0.4717230834202142</v>
+        <v>0.6072822297795264</v>
       </c>
       <c r="L10" s="11" t="n">
-        <v>0.3454285520418154</v>
+        <v>0.4676285534459973</v>
       </c>
       <c r="M10" s="11" t="n">
-        <v>0.2257505536938685</v>
+        <v>0.3347250015924711</v>
       </c>
       <c r="N10" s="11" t="n">
-        <v>0.1047557192049378</v>
+        <v>0.2033203886465199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>